<commit_message>
Update training/test results spreadsheet
</commit_message>
<xml_diff>
--- a/cm/training_results_history.xlsx
+++ b/cm/training_results_history.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -882,6 +882,46 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-13 12:08:17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baseline </t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>U-Net (ResNet34 encoder)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>39</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1958</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9414</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.9467</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.9439</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.8938</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Baseline for reference</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add latest training results
</commit_message>
<xml_diff>
--- a/cm/training_results_history.xlsx
+++ b/cm/training_results_history.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -922,6 +922,46 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-14 23:24:44</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>lower_epochs_1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DeepLabV3_ResNet50</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.9025</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.9088000000000001</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.8342000000000001</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>20 epochs using lr=2e-5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>